<commit_message>
Adopt neutral tone across project text
</commit_message>
<xml_diff>
--- a/docs/reference/data-dictionary.xlsx
+++ b/docs/reference/data-dictionary.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data dictionary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -507,12 +507,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How to use it</t>
+          <t>Entry structure</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start with “What it is”, “How it works”, and “How to read it”. Use “Exact source” when checking the XML.</t>
+          <t>Each entry contains Definition, Calculation, Interpretation, and Empty-value meaning. Exact source identifies XML provenance.</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -649,22 +649,22 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>What it is</t>
+          <t>Definition</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>How it works</t>
+          <t>Calculation</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>How to read it</t>
+          <t>Interpretation</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>Empty value meaning</t>
+          <t>Empty-value meaning</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Use this value to keep communities separate. Each Stack Exchange site has its own topics, users, and moderation practices.</t>
+          <t>The value distinguishes communities because each Stack Exchange site has its own topics, accounts, and moderation practices.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Treat every snapshot-based score, view, count, and text field as observed by this date. It defines the end of the observation period.</t>
+          <t>Every snapshot-based score, view, count, and text field is observed by this date, which defines the end of the observation period.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Use this stable number to join records and find the same question in extracts and tables.</t>
+          <t>The stable number supports record joins and identifies the same question across extracts and tables.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Open this address to inspect the public question page when it remains available online.</t>
+          <t>The address identifies the public question page when that page remains available online.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Use this timestamp to place the question in a period or cohort. Stack Exchange dump timestamps are recorded in UTC.</t>
+          <t>The timestamp places the question in a period or cohort. Stack Exchange dump timestamps are recorded in UTC.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Compare it with the creation time. A later timestamp shows that an edit occurred and gives the most recent recorded edit time.</t>
+          <t>Comparison with the creation time identifies whether an edit occurred and gives the most recent recorded edit time.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Read it as the short wording shown above the question body in the dump snapshot.</t>
+          <t>The value is the short wording displayed above the question body in the dump snapshot.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Use it when rendered formatting, code blocks, links, and images must be preserved. HTML-aware software is required for display.</t>
+          <t>The value preserves rendered formatting, code blocks, links, and images. Display requires HTML-aware software.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Parse the HTML and join visible text with normalized spaces.</t>
+          <t>The HTML is parsed, and visible text is joined with normalized spaces.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Use it for reading and text processing. Formatting is flattened into spaces while visible code text remains present.</t>
+          <t>The value supports reading and text processing. Formatting is flattened into spaces while visible code text remains present.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Use it for source verification. Each tag appears between angle brackets, following the original dump notation.</t>
+          <t>The value supports source verification. Each tag appears between angle brackets in the original dump notation.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Extract each name between angle brackets and join the names with semicolons.</t>
+          <t>Each name between angle brackets is extracted, and the names are joined with semicolons.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Split this value at semicolons to obtain individual topic names. One question can carry several tags.</t>
+          <t>Semicolon separation yields the individual topic names. One question can carry several tags.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Use this licence together with the question URL and author information when sharing or reusing question content.</t>
+          <t>The licence, question URL, and author information govern sharing and reuse of question content.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier for attribution and source joins when the author account is available.</t>
+          <t>The identifier supports attribution and source joins when the author account is available.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Use this source name for attribution when Stack Exchange stores a name directly on the post.</t>
+          <t>The source name supports attribution when Stack Exchange stores a name directly on the post.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Read zero as no answer in the platform-maintained count. Compare this field with available_answer_count to identify source-row differences.</t>
+          <t>Zero denotes no answer in the platform-maintained count. Comparison with available_answer_count identifies source-row differences.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Read zero as no question comment in the platform-maintained count. Compare it with available_question_comment_count to identify source-row differences.</t>
+          <t>Zero denotes no question comment in the platform-maintained count. Comparison with available_question_comment_count identifies source-row differences.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>A present value means that the author selected an answer as the solution. Use the identifier to locate that answer row.</t>
+          <t>A present value means that the author selected an answer as the solution. The identifier locates that answer row.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Remove preformatted and code elements, extract visible prose, and count Unicode word tokens.</t>
+          <t>Preformatted and code elements are removed before visible-prose extraction and Unicode word-token counting.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Larger values mean longer prose. Use length together with content and response evidence during difficulty analysis.</t>
+          <t>Larger values mean longer prose. Question length combines with content and response evidence during difficulty analysis.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Extract each pre element and count its non-empty text lines.</t>
+          <t>Each pre element is extracted, and its non-empty text lines are counted.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Count HTML a elements that contain an href attribute.</t>
+          <t>The value equals the number of HTML a elements containing an href attribute.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Count HTML img elements.</t>
+          <t>The value equals the number of HTML img elements.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2204,12 +2204,12 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Count the parsed tag names.</t>
+          <t>The value equals the number of parsed tag names.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>This is usually between one and the site tag limit. Larger values describe a question assigned to more topics.</t>
+          <t>The value is usually between one and the site tag limit. Larger values describe a question assigned to more topics.</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Count matching PostTypeId = 2 rows in the dump.</t>
+          <t>The value equals the number of matching PostTypeId = 2 rows in the dump.</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Sort available answers by CreationDate and numeric Id, then select the first row.</t>
+          <t>Available answers are ordered by CreationDate and numeric Id; the first row supplies the value.</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier to locate the earliest available answer selected by timestamp and numeric ID.</t>
+          <t>The identifier locates the earliest available answer selected by timestamp and numeric ID.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2452,12 +2452,12 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Take CreationDate from first_answer_id.</t>
+          <t>The value is the CreationDate associated with first_answer_id.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Compare it with the question creation time to see when the first available answer appeared.</t>
+          <t>Comparison with the question creation time shows when the first available answer appeared.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Calculate every non-negative answer posting delay and take the median.</t>
+          <t>The value is the median of all non-negative answer-posting delays.</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Take CreationDate from the available accepted-answer row.</t>
+          <t>The value is the CreationDate from the available accepted-answer row.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>This is the posting time of the answer that is currently accepted. It records answer arrival and serves as the start point for that answer content.</t>
+          <t>The value is the posting time of the answer that is currently accepted. It records answer arrival and serves as the start point for that answer content.</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Build https://{site}/a/{accepted_answer_id}.</t>
+          <t>The address is constructed as https://{site}/a/{accepted_answer_id}.</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Open this address to inspect and attribute the accepted answer when it remains available online.</t>
+          <t>The address identifies the currently accepted answer and supports attribution when that page remains available online.</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier for accepted-answer author attribution and source joins when the account is available.</t>
+          <t>The identifier supports accepted-answer author attribution and source joins when the account is available.</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Use this source name for accepted-answer attribution when Stack Exchange stores it directly on the answer row.</t>
+          <t>The source name supports accepted-answer attribution when Stack Exchange stores it directly on the answer row.</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Use this licence together with the accepted-answer URL and author information when sharing or reusing answer content.</t>
+          <t>The licence, accepted-answer URL, and author information govern sharing and reuse of answer content.</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Select the earliest matching VoteTypeId = 1 date. Vote timestamps have day-level precision in the public dump.</t>
+          <t>The earliest matching VoteTypeId = 1 date supplies the value. Public-dump vote timestamps have day-level precision.</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -3258,12 +3258,12 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Parse the accepted answer HTML and join visible text with normalized spaces.</t>
+          <t>The accepted-answer HTML is parsed, and visible text is joined with normalized spaces.</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Read this as the visible accepted-answer content with HTML formatting flattened into spaces.</t>
+          <t>The value is the visible accepted-answer content with HTML formatting flattened into spaces.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Count matching question-comment rows; comments on answers are outside the agreed extraction scope.</t>
+          <t>The value equals the number of matching question-comment rows; comments on answers are outside the agreed extraction scope.</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Count question comments whose CreationDate is earlier than first_answer_creation_datetime.</t>
+          <t>The value equals the number of question comments whose CreationDate precedes first_answer_creation_datetime.</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Larger values give the question more time to accumulate answers, comments, votes, and views. Use this field to control unequal follow-up time.</t>
+          <t>Larger values provide more time for accumulated answers, comments, votes, and views. The field controls unequal follow-up time.</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Adopt neutral tone across project text (#11)
Maintained authored surfaces now use impersonal, descriptive language while source data and executable behavior remain unchanged.
</commit_message>
<xml_diff>
--- a/docs/reference/data-dictionary.xlsx
+++ b/docs/reference/data-dictionary.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data dictionary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -507,12 +507,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How to use it</t>
+          <t>Entry structure</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start with “What it is”, “How it works”, and “How to read it”. Use “Exact source” when checking the XML.</t>
+          <t>Each entry contains Definition, Calculation, Interpretation, and Empty-value meaning. Exact source identifies XML provenance.</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -649,22 +649,22 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>What it is</t>
+          <t>Definition</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>How it works</t>
+          <t>Calculation</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>How to read it</t>
+          <t>Interpretation</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>Empty value meaning</t>
+          <t>Empty-value meaning</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Use this value to keep communities separate. Each Stack Exchange site has its own topics, users, and moderation practices.</t>
+          <t>The value distinguishes communities because each Stack Exchange site has its own topics, accounts, and moderation practices.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Treat every snapshot-based score, view, count, and text field as observed by this date. It defines the end of the observation period.</t>
+          <t>Every snapshot-based score, view, count, and text field is observed by this date, which defines the end of the observation period.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Use this stable number to join records and find the same question in extracts and tables.</t>
+          <t>The stable number supports record joins and identifies the same question across extracts and tables.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Open this address to inspect the public question page when it remains available online.</t>
+          <t>The address identifies the public question page when that page remains available online.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Use this timestamp to place the question in a period or cohort. Stack Exchange dump timestamps are recorded in UTC.</t>
+          <t>The timestamp places the question in a period or cohort. Stack Exchange dump timestamps are recorded in UTC.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Compare it with the creation time. A later timestamp shows that an edit occurred and gives the most recent recorded edit time.</t>
+          <t>Comparison with the creation time identifies whether an edit occurred and gives the most recent recorded edit time.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Read it as the short wording shown above the question body in the dump snapshot.</t>
+          <t>The value is the short wording displayed above the question body in the dump snapshot.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Use it when rendered formatting, code blocks, links, and images must be preserved. HTML-aware software is required for display.</t>
+          <t>The value preserves rendered formatting, code blocks, links, and images. Display requires HTML-aware software.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Parse the HTML and join visible text with normalized spaces.</t>
+          <t>The HTML is parsed, and visible text is joined with normalized spaces.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Use it for reading and text processing. Formatting is flattened into spaces while visible code text remains present.</t>
+          <t>The value supports reading and text processing. Formatting is flattened into spaces while visible code text remains present.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Use it for source verification. Each tag appears between angle brackets, following the original dump notation.</t>
+          <t>The value supports source verification. Each tag appears between angle brackets in the original dump notation.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Extract each name between angle brackets and join the names with semicolons.</t>
+          <t>Each name between angle brackets is extracted, and the names are joined with semicolons.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Split this value at semicolons to obtain individual topic names. One question can carry several tags.</t>
+          <t>Semicolon separation yields the individual topic names. One question can carry several tags.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Use this licence together with the question URL and author information when sharing or reusing question content.</t>
+          <t>The licence, question URL, and author information govern sharing and reuse of question content.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier for attribution and source joins when the author account is available.</t>
+          <t>The identifier supports attribution and source joins when the author account is available.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Use this source name for attribution when Stack Exchange stores a name directly on the post.</t>
+          <t>The source name supports attribution when Stack Exchange stores a name directly on the post.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Read zero as no answer in the platform-maintained count. Compare this field with available_answer_count to identify source-row differences.</t>
+          <t>Zero denotes no answer in the platform-maintained count. Comparison with available_answer_count identifies source-row differences.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Read zero as no question comment in the platform-maintained count. Compare it with available_question_comment_count to identify source-row differences.</t>
+          <t>Zero denotes no question comment in the platform-maintained count. Comparison with available_question_comment_count identifies source-row differences.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>A present value means that the author selected an answer as the solution. Use the identifier to locate that answer row.</t>
+          <t>A present value means that the author selected an answer as the solution. The identifier locates that answer row.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Remove preformatted and code elements, extract visible prose, and count Unicode word tokens.</t>
+          <t>Preformatted and code elements are removed before visible-prose extraction and Unicode word-token counting.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Larger values mean longer prose. Use length together with content and response evidence during difficulty analysis.</t>
+          <t>Larger values mean longer prose. Question length combines with content and response evidence during difficulty analysis.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Extract each pre element and count its non-empty text lines.</t>
+          <t>Each pre element is extracted, and its non-empty text lines are counted.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Count HTML a elements that contain an href attribute.</t>
+          <t>The value equals the number of HTML a elements containing an href attribute.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Count HTML img elements.</t>
+          <t>The value equals the number of HTML img elements.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2204,12 +2204,12 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Count the parsed tag names.</t>
+          <t>The value equals the number of parsed tag names.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>This is usually between one and the site tag limit. Larger values describe a question assigned to more topics.</t>
+          <t>The value is usually between one and the site tag limit. Larger values describe a question assigned to more topics.</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Count matching PostTypeId = 2 rows in the dump.</t>
+          <t>The value equals the number of matching PostTypeId = 2 rows in the dump.</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Sort available answers by CreationDate and numeric Id, then select the first row.</t>
+          <t>Available answers are ordered by CreationDate and numeric Id; the first row supplies the value.</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier to locate the earliest available answer selected by timestamp and numeric ID.</t>
+          <t>The identifier locates the earliest available answer selected by timestamp and numeric ID.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2452,12 +2452,12 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Take CreationDate from first_answer_id.</t>
+          <t>The value is the CreationDate associated with first_answer_id.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Compare it with the question creation time to see when the first available answer appeared.</t>
+          <t>Comparison with the question creation time shows when the first available answer appeared.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Calculate every non-negative answer posting delay and take the median.</t>
+          <t>The value is the median of all non-negative answer-posting delays.</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Take CreationDate from the available accepted-answer row.</t>
+          <t>The value is the CreationDate from the available accepted-answer row.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>This is the posting time of the answer that is currently accepted. It records answer arrival and serves as the start point for that answer content.</t>
+          <t>The value is the posting time of the answer that is currently accepted. It records answer arrival and serves as the start point for that answer content.</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Build https://{site}/a/{accepted_answer_id}.</t>
+          <t>The address is constructed as https://{site}/a/{accepted_answer_id}.</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Open this address to inspect and attribute the accepted answer when it remains available online.</t>
+          <t>The address identifies the currently accepted answer and supports attribution when that page remains available online.</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Use this identifier for accepted-answer author attribution and source joins when the account is available.</t>
+          <t>The identifier supports accepted-answer author attribution and source joins when the account is available.</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Use this source name for accepted-answer attribution when Stack Exchange stores it directly on the answer row.</t>
+          <t>The source name supports accepted-answer attribution when Stack Exchange stores it directly on the answer row.</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Use this licence together with the accepted-answer URL and author information when sharing or reusing answer content.</t>
+          <t>The licence, accepted-answer URL, and author information govern sharing and reuse of answer content.</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Select the earliest matching VoteTypeId = 1 date. Vote timestamps have day-level precision in the public dump.</t>
+          <t>The earliest matching VoteTypeId = 1 date supplies the value. Public-dump vote timestamps have day-level precision.</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -3258,12 +3258,12 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Parse the accepted answer HTML and join visible text with normalized spaces.</t>
+          <t>The accepted-answer HTML is parsed, and visible text is joined with normalized spaces.</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Read this as the visible accepted-answer content with HTML formatting flattened into spaces.</t>
+          <t>The value is the visible accepted-answer content with HTML formatting flattened into spaces.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Count matching question-comment rows; comments on answers are outside the agreed extraction scope.</t>
+          <t>The value equals the number of matching question-comment rows; comments on answers are outside the agreed extraction scope.</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Count question comments whose CreationDate is earlier than first_answer_creation_datetime.</t>
+          <t>The value equals the number of question comments whose CreationDate precedes first_answer_creation_datetime.</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Calculated by us</t>
+          <t>Calculated by project</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Larger values give the question more time to accumulate answers, comments, votes, and views. Use this field to control unequal follow-up time.</t>
+          <t>Larger values provide more time for accumulated answers, comments, votes, and views. The field controls unequal follow-up time.</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">

</xml_diff>